<commit_message>
Từ điển: thêm băng dính/keo → páska (+ 2 mặt, điện, giấy, đóng gói)
10 mục: bang dinh/bang keo/bang dan → paska; băng keo hai mặt → oboustranná
páska; băng keo điện → izolační páska; băng keo giấy → malířská páska; băng
keo đóng gói → balicí páska. dict 633 mục. v1.5.9.9.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tudien.xlsx
+++ b/tudien.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tu dien Viet-Sec" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tu dien Viet-Sec" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D566"/>
+  <dimension ref="A1:D576"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -12884,6 +12884,226 @@
         </is>
       </c>
     </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>bang dinh</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>băng dính</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>páska</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>bang keo</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>băng keo</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>páska</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>bang dan</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>băng dán</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>páska</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>bang dinh trong</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>băng dính trong</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>lepicí páska</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>bang keo dong goi</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>băng keo đóng gói</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>balicí páska</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>bang keo hai mat</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>băng keo hai mặt</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>oboustranná páska</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>bang dinh hai mat</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>băng dính hai mặt</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>oboustranná páska</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>bang keo dien</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>băng keo điện</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>izolační páska</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>bang dinh dien</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>băng dính điện</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>izolační páska</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>bang keo giay</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>băng keo giấy</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>malířská páska</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>